<commit_message>
Added batch module changes
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/Team5Data.xlsx
+++ b/src/test/resources/testData/Team5Data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mahaj\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sudhi\IdeaProjects\APITesters_Team05\src\test\resources\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39372372-FB7D-4C2D-9EA5-00569BC9D9E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17D83EB8-95B5-4D45-8EEF-24BFF3D3E1D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{E075535D-C164-41C6-889D-32DAEADAA696}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="5" activeTab="8" xr2:uid="{E075535D-C164-41C6-889D-32DAEADAA696}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="8" r:id="rId1"/>
@@ -18,9 +18,10 @@
     <sheet name="ForgotPassword" sheetId="9" r:id="rId3"/>
     <sheet name="CreateProgram" sheetId="2" r:id="rId4"/>
     <sheet name="ProgramSetupsheetname" sheetId="7" r:id="rId5"/>
-    <sheet name="Sheet4" sheetId="11" r:id="rId6"/>
+    <sheet name="UpdateBatchbyBatchId" sheetId="11" r:id="rId6"/>
     <sheet name="UpdateProgramById" sheetId="3" r:id="rId7"/>
     <sheet name="UpdateProgramByName" sheetId="6" r:id="rId8"/>
+    <sheet name="CreateBatch" sheetId="14" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -32,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="176">
   <si>
     <t>Scenario</t>
   </si>
@@ -187,36 +188,6 @@
     <t>TimeTravel</t>
   </si>
   <si>
-    <t>Live on Mars safelyab</t>
-  </si>
-  <si>
-    <t>MarsLifePrepab</t>
-  </si>
-  <si>
-    <t>StarVoyagersab</t>
-  </si>
-  <si>
-    <t>Fight to surviveab</t>
-  </si>
-  <si>
-    <t>BattleArenaab</t>
-  </si>
-  <si>
-    <t>Care for unicornab</t>
-  </si>
-  <si>
-    <t>UnicornCareab</t>
-  </si>
-  <si>
-    <t>Delete test id caseab</t>
-  </si>
-  <si>
-    <t>DeleteByIdDragonab</t>
-  </si>
-  <si>
-    <t>DeleteNamePhoenix</t>
-  </si>
-  <si>
     <t>ScenarioType</t>
   </si>
   <si>
@@ -313,20 +284,290 @@
     <t>Test05gmail.com</t>
   </si>
   <si>
-    <t>TeamFive@124</t>
-  </si>
-  <si>
-    <t>TeamFive@200</t>
-  </si>
-  <si>
-    <t>TeamFive@281</t>
+    <t>batchDescription</t>
+  </si>
+  <si>
+    <t>batchName</t>
+  </si>
+  <si>
+    <t>batchNoOfClasses</t>
+  </si>
+  <si>
+    <t>batchStatus</t>
+  </si>
+  <si>
+    <t>programId</t>
+  </si>
+  <si>
+    <t>Admin creates batch with a program name that does not match the associated program id</t>
+  </si>
+  <si>
+    <t>test-abc</t>
+  </si>
+  <si>
+    <t>Amindb testing</t>
+  </si>
+  <si>
+    <t>Admin creates batch without underscore format in batch name</t>
+  </si>
+  <si>
+    <t>test-ab</t>
+  </si>
+  <si>
+    <t>Admin creates batch with hyphen format in batch name</t>
+  </si>
+  <si>
+    <t>Admin creates batch with characters in the suffix of batch name</t>
+  </si>
+  <si>
+    <t>Amindb testing_AB</t>
+  </si>
+  <si>
+    <t>Admin creates batch with special characters in the suffix of batch name</t>
+  </si>
+  <si>
+    <t>Amindb testing_#$</t>
+  </si>
+  <si>
+    <t>Admin creates batch with batch name length more than 28 characters in total</t>
+  </si>
+  <si>
+    <t>Amindqwertyuioplkjhgfdsazxcvbn</t>
+  </si>
+  <si>
+    <t>Admin creates batch with batch name length less than 6 characters in total</t>
+  </si>
+  <si>
+    <t>Amind</t>
+  </si>
+  <si>
+    <t>Admin creates batch with duplicate batch name</t>
+  </si>
+  <si>
+    <t>Admin creates batch with batch description less than 4 characters</t>
+  </si>
+  <si>
+    <t>Admin creates batch with batch description more than 25 characters</t>
+  </si>
+  <si>
+    <t>Admin creates batch with random characters in status field</t>
+  </si>
+  <si>
+    <t>random</t>
+  </si>
+  <si>
+    <t>Admin creates batch with random numbers in status field</t>
+  </si>
+  <si>
+    <t>Admin creates batch with special characters in status field</t>
+  </si>
+  <si>
+    <t>$#&amp;</t>
+  </si>
+  <si>
+    <t>Admin creates batch with non numeric value in number of classes</t>
+  </si>
+  <si>
+    <t>aa</t>
+  </si>
+  <si>
+    <t>Admin creates batch with number of classes length less than 1</t>
+  </si>
+  <si>
+    <t>Admin creates batch with number of classes length more than 99</t>
+  </si>
+  <si>
+    <t>Admin creates batch with inactive program ID</t>
+  </si>
+  <si>
+    <t>Joyful learning_120</t>
+  </si>
+  <si>
+    <t>Joyful learning</t>
+  </si>
+  <si>
+    <t>Admin creates batch with program that is not exist in the system</t>
+  </si>
+  <si>
+    <t>Amindbtesting_120</t>
+  </si>
+  <si>
+    <t>Admin creates batch with invalid endpoint</t>
+  </si>
+  <si>
+    <t>Admin creates batch with invalid method</t>
+  </si>
+  <si>
+    <t>Admin creates a batch with invalid token</t>
+  </si>
+  <si>
+    <t>Admin creates batch with only mandatory fields</t>
+  </si>
+  <si>
+    <t>Admin creates batch with both mandatory and optional fields</t>
+  </si>
+  <si>
+    <t>Admin creates batch with only optional fields</t>
+  </si>
+  <si>
+    <t>bat</t>
+  </si>
+  <si>
+    <t>LongesssssssssstbatchDescription</t>
+  </si>
+  <si>
+    <t>Admin updates a batch by batch id with missing mandatory fields in request body</t>
+  </si>
+  <si>
+    <t>Admin updates a batch by batch id with duplicate batch name</t>
+  </si>
+  <si>
+    <t>Admin updates a batch by batch id with invalid batch name format</t>
+  </si>
+  <si>
+    <t>Admin updates a batch by batch id with batch name more than allowable length</t>
+  </si>
+  <si>
+    <t>Admin updates a batch by batch id with batch name less than allowable length in total</t>
+  </si>
+  <si>
+    <t>Admin updates a batch by batch id with invalid batch description</t>
+  </si>
+  <si>
+    <t>Admin updates a batch by batch id with invalid batch status</t>
+  </si>
+  <si>
+    <t>Admin updates a batch by batch id with invalid batch number of classes</t>
+  </si>
+  <si>
+    <t>Admin updates a batch by batch id with invalid program id</t>
+  </si>
+  <si>
+    <t>Admin updates a batch by batch id with special characters in program name</t>
+  </si>
+  <si>
+    <t>Admin updates a batch by batch id with numbers in program name</t>
+  </si>
+  <si>
+    <t>Admin updates a batch by batch id with a program name that does not match the associated program id</t>
+  </si>
+  <si>
+    <t>Admin updates a batch by batch id with inactive program</t>
+  </si>
+  <si>
+    <t>Admin updates a batch by batch id with invalid endpoint</t>
+  </si>
+  <si>
+    <t>Admin updates a batch by batch id with invalid method</t>
+  </si>
+  <si>
+    <t>Admin updates a batch with invalid batch ID</t>
+  </si>
+  <si>
+    <t>Admin updates a batch with valid batch ID</t>
+  </si>
+  <si>
+    <t>updatedescription</t>
+  </si>
+  <si>
+    <t>Amindb testing_12</t>
+  </si>
+  <si>
+    <t>Amindb testing12</t>
+  </si>
+  <si>
+    <t>Amindb testingqwertfdsacvhyb_12</t>
+  </si>
+  <si>
+    <t>Am_12</t>
+  </si>
+  <si>
+    <t>updatedesc@#$</t>
+  </si>
+  <si>
+    <t>Amindb testing_98</t>
+  </si>
+  <si>
+    <t>200 ok bug</t>
+  </si>
+  <si>
+    <t>Amindb testing_3</t>
+  </si>
+  <si>
+    <t>Joyful learning_23</t>
+  </si>
+  <si>
+    <t>Admin updates a batch by batch id with invalid token</t>
+  </si>
+  <si>
+    <t>Amindb testing_38</t>
+  </si>
+  <si>
+    <t>speci&amp;l#@$</t>
+  </si>
+  <si>
+    <t>bug</t>
+  </si>
+  <si>
+    <t>200 ok bug update with associate pgm name of pgm id</t>
+  </si>
+  <si>
+    <t>TeamFive@123</t>
+  </si>
+  <si>
+    <t>TeamFive@125</t>
+  </si>
+  <si>
+    <t>Valid Email</t>
+  </si>
+  <si>
+    <t>Live on Mars safelyop</t>
+  </si>
+  <si>
+    <t>MarsLifePrepop</t>
+  </si>
+  <si>
+    <t>StarVoyagersop</t>
+  </si>
+  <si>
+    <t>BattleArenaop</t>
+  </si>
+  <si>
+    <t>Fight to surviveop</t>
+  </si>
+  <si>
+    <t>Amindb Testsop</t>
+  </si>
+  <si>
+    <t>Care for unicornop</t>
+  </si>
+  <si>
+    <t>UnicornCareop</t>
+  </si>
+  <si>
+    <t>DeleteNamePhoenixop</t>
+  </si>
+  <si>
+    <t>Delete test id caseop</t>
+  </si>
+  <si>
+    <t>DeleteByIdDragonop</t>
+  </si>
+  <si>
+    <t>test-abc_18</t>
+  </si>
+  <si>
+    <t>test-ab78</t>
+  </si>
+  <si>
+    <t>test-ab_38</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -357,8 +598,25 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="7"/>
+      <color rgb="FF0451A5"/>
+      <name val="Courier New"/>
+      <family val="3"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -371,8 +629,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -410,12 +674,23 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -430,6 +705,24 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -449,9 +742,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -489,7 +782,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -595,7 +888,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -737,7 +1030,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -745,185 +1038,188 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5870DA65-7A89-41DE-8F09-CF478CA71B5C}">
-  <dimension ref="A1:D13"/>
-  <sheetFormatPr defaultColWidth="22.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:E13"/>
+  <sheetFormatPr defaultColWidth="22.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="12" t="s">
+        <v>160</v>
+      </c>
+      <c r="D2" s="3">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>160</v>
+      </c>
+      <c r="D3" s="3">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>160</v>
+      </c>
+      <c r="D4" s="3">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C5" s="12" t="s">
+        <v>160</v>
+      </c>
+      <c r="D5" s="3">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="B6" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="C6" s="12" t="s">
+        <v>160</v>
+      </c>
+      <c r="D6" s="3">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="D2" s="3">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="D3" s="3">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="D4" s="3">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="D5" s="3">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="B6" s="4" t="s">
+      <c r="B7" s="4" t="s">
         <v>73</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="D6" s="3">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>83</v>
       </c>
       <c r="C7" s="3"/>
       <c r="D7" s="3">
         <v>400</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="D8" s="3">
         <v>401</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E8" s="11" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="D9" s="3">
         <v>400</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="C10" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="D10" s="3">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>160</v>
+      </c>
+      <c r="D11" s="3">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="D10" s="3">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A11" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="D11" s="3">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" s="3" t="s">
-        <v>81</v>
-      </c>
       <c r="B12" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>93</v>
+        <v>73</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>160</v>
       </c>
       <c r="D12" s="3">
         <v>405</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>93</v>
+        <v>73</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>160</v>
       </c>
       <c r="D13" s="3">
-        <v>404</v>
+        <v>401</v>
       </c>
     </row>
   </sheetData>
@@ -931,12 +1227,19 @@
     <hyperlink ref="B6" r:id="rId1" display="mailto:notfound@mail.com" xr:uid="{943820FE-FD16-4AE9-9F4B-54ED6D6CE8CC}"/>
     <hyperlink ref="B7" r:id="rId2" xr:uid="{0E75F417-5043-4022-A096-BA61737FD3B2}"/>
     <hyperlink ref="B11" r:id="rId3" display="mailto:inactive@mail.com" xr:uid="{738D5541-8B9E-4C87-B264-89C50A83D259}"/>
-    <hyperlink ref="C5" r:id="rId4" xr:uid="{3754E669-C712-477D-AC77-5C63D6807900}"/>
-    <hyperlink ref="B8" r:id="rId5" xr:uid="{E0301111-1FE5-4FC8-8B29-717CAEAEA29F}"/>
-    <hyperlink ref="B9" r:id="rId6" xr:uid="{B14CBF5D-8073-4C72-AA9B-3A52D893A42D}"/>
-    <hyperlink ref="B10" r:id="rId7" xr:uid="{D6942936-5D52-4C4A-8ECA-9DE8722DC4E7}"/>
-    <hyperlink ref="B12" r:id="rId8" xr:uid="{3C895F9A-5852-422F-BA70-9072953C0F79}"/>
-    <hyperlink ref="B13" r:id="rId9" xr:uid="{76EFE8C1-C1B1-43B2-BA64-14F7AC4BAF9C}"/>
+    <hyperlink ref="B8" r:id="rId4" xr:uid="{E0301111-1FE5-4FC8-8B29-717CAEAEA29F}"/>
+    <hyperlink ref="B9" r:id="rId5" xr:uid="{B14CBF5D-8073-4C72-AA9B-3A52D893A42D}"/>
+    <hyperlink ref="B10" r:id="rId6" xr:uid="{D6942936-5D52-4C4A-8ECA-9DE8722DC4E7}"/>
+    <hyperlink ref="B12" r:id="rId7" xr:uid="{3C895F9A-5852-422F-BA70-9072953C0F79}"/>
+    <hyperlink ref="B13" r:id="rId8" xr:uid="{76EFE8C1-C1B1-43B2-BA64-14F7AC4BAF9C}"/>
+    <hyperlink ref="C2" r:id="rId9" xr:uid="{127FD2B5-78BB-464B-A9CD-CD008DC6CD93}"/>
+    <hyperlink ref="C3" r:id="rId10" xr:uid="{8DF09848-83DE-4BBF-B1A2-1AEEA19B4346}"/>
+    <hyperlink ref="C4" r:id="rId11" xr:uid="{19881271-15CD-4524-88E0-7E1A48BEE6D7}"/>
+    <hyperlink ref="C5" r:id="rId12" xr:uid="{31DDF559-C92D-4E93-A112-5CF6787C9F78}"/>
+    <hyperlink ref="C6" r:id="rId13" xr:uid="{485AF9D4-F737-467E-9B83-4DE2D7921067}"/>
+    <hyperlink ref="C11" r:id="rId14" xr:uid="{E9BE5A0B-436B-4C8D-A311-75820BD6C958}"/>
+    <hyperlink ref="C12" r:id="rId15" xr:uid="{6642A2F1-B387-4F6D-8494-366A09C46D80}"/>
+    <hyperlink ref="C13" r:id="rId16" xr:uid="{1156645C-D24C-4677-A8E8-4489D07A92B0}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -945,113 +1248,113 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{443B2256-BF49-449E-9DD1-4030FF98AED6}">
   <dimension ref="A1:D9"/>
-  <sheetFormatPr defaultColWidth="27.36328125" defaultRowHeight="38.5" customHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="27.33203125" defaultRowHeight="38.549999999999997" customHeight="1" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:4" ht="38.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" ht="38.549999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="38.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="38.549999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>95</v>
+        <v>159</v>
       </c>
       <c r="D2" s="3">
         <v>200</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="38.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" ht="38.549999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>94</v>
+        <v>159</v>
       </c>
       <c r="D3" s="3">
         <v>400</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="38.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" ht="38.549999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="D4" s="3">
         <v>400</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="38.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" ht="38.549999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>94</v>
+        <v>159</v>
       </c>
       <c r="D5" s="3">
         <v>404</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="38.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" ht="38.549999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>94</v>
+        <v>159</v>
       </c>
       <c r="D6" s="3">
         <v>405</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="38.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" ht="38.549999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>94</v>
+        <v>159</v>
       </c>
       <c r="D7" s="3">
         <v>401</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="38.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" ht="38.549999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3"/>
       <c r="B8" s="4"/>
       <c r="C8" s="3"/>
       <c r="D8" s="3"/>
     </row>
-    <row r="9" spans="1:4" ht="38.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" ht="38.549999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -1066,11 +1369,11 @@
     <hyperlink ref="B5" r:id="rId5" xr:uid="{146FF6F4-CFA0-4965-BB12-16ED707B7AFF}"/>
     <hyperlink ref="B6" r:id="rId6" xr:uid="{C10FE077-11C5-4888-85F2-476E58BD487E}"/>
     <hyperlink ref="B7" r:id="rId7" xr:uid="{34847948-15D7-4525-A5B9-0610F9EDA075}"/>
-    <hyperlink ref="C2" r:id="rId8" xr:uid="{8DA12DBD-CA8B-47BE-AEDF-95E5B00491BD}"/>
-    <hyperlink ref="C3" r:id="rId9" xr:uid="{9DE0BC97-2654-4FEE-9A7D-6C347051C977}"/>
-    <hyperlink ref="C5" r:id="rId10" xr:uid="{9E26EEA7-4001-4DB8-A422-E287297ED374}"/>
-    <hyperlink ref="C6" r:id="rId11" xr:uid="{9D1B9DFD-0ECC-4E2C-86AD-086BDD8020F8}"/>
-    <hyperlink ref="C7" r:id="rId12" xr:uid="{B9591C4B-D394-420B-80C9-D698E09C7577}"/>
+    <hyperlink ref="C2" r:id="rId8" xr:uid="{D5776F13-F123-4867-B73F-0FD7E5F4C73B}"/>
+    <hyperlink ref="C3" r:id="rId9" xr:uid="{D352CC11-255C-46C6-982D-C549B1581CEF}"/>
+    <hyperlink ref="C5" r:id="rId10" xr:uid="{9CA76A89-3119-49B8-BB35-B0EF3178D561}"/>
+    <hyperlink ref="C6" r:id="rId11" xr:uid="{06BEA948-B30F-4124-AEC4-D20FF720AF46}"/>
+    <hyperlink ref="C7" r:id="rId12" xr:uid="{AE33B4A3-38EB-4675-B6BD-F9375CD09E48}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1079,107 +1382,113 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FC4AC91-F305-4600-B058-9746246064A0}">
   <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultColWidth="28.36328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="28.33203125" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="19.26953125" customWidth="1"/>
+    <col min="3" max="3" width="19.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="B2" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="C2">
         <v>405</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="C3">
         <v>404</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="3">
         <v>400</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="C5" s="3">
         <v>400</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="C6" s="3">
         <v>400</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="B7" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="C7" s="3">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="B8" s="13" t="s">
         <v>73</v>
       </c>
-      <c r="C7" s="3">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A8" s="3"/>
-      <c r="B8" s="4"/>
-      <c r="C8" s="3"/>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C8" s="3">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="3"/>
       <c r="B9" s="4"/>
       <c r="C9" s="3"/>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="3"/>
       <c r="B10" s="4"/>
       <c r="C10" s="3"/>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="3"/>
       <c r="B11" s="4"/>
       <c r="C11" s="3"/>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="3"/>
       <c r="B12" s="4"/>
       <c r="C12" s="3"/>
@@ -1196,17 +1505,17 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51118034-34E5-45E2-A5A5-3C55CA0A81A2}">
   <dimension ref="A1:E15"/>
-  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="81.08984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.6328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.6328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.81640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.1796875" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="8.90625" style="1"/>
+    <col min="1" max="1" width="81.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1223,7 +1532,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>24</v>
       </c>
@@ -1237,7 +1546,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
@@ -1251,7 +1560,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>11</v>
       </c>
@@ -1265,7 +1574,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>12</v>
       </c>
@@ -1279,7 +1588,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
@@ -1293,7 +1602,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>17</v>
       </c>
@@ -1307,7 +1616,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>19</v>
       </c>
@@ -1315,7 +1624,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>20</v>
       </c>
@@ -1332,7 +1641,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>22</v>
       </c>
@@ -1349,15 +1658,15 @@
         <v>400</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>51</v>
+        <v>162</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>52</v>
+        <v>163</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>6</v>
@@ -1366,12 +1675,12 @@
         <v>201</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>53</v>
+        <v>164</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>6</v>
@@ -1380,7 +1689,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>25</v>
       </c>
@@ -1397,7 +1706,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>26</v>
       </c>
@@ -1414,7 +1723,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>27</v>
       </c>
@@ -1442,17 +1751,17 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9CC793A-8931-401A-A548-6DE35F95950D}">
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.08984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.6328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.453125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.81640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.1796875" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="8.90625" style="1"/>
+    <col min="1" max="1" width="20.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1469,15 +1778,15 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>44</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>54</v>
+        <v>166</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>55</v>
+        <v>165</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>6</v>
@@ -1493,27 +1802,434 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D8C71BF-CB4E-4334-8784-890AB6A8A9AA}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
+  <dimension ref="A1:I19"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="92.6640625" style="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.6640625" style="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="29.33203125" style="7" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.5546875" style="7" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.88671875" style="7" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.109375" style="7" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.5546875" style="7" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.44140625" style="7" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="8.88671875" style="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1" s="7" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A2" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="D2" s="7">
+        <v>56</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="H2" s="7">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A3" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="H3" s="7">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="D4" s="7">
+        <v>32</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="H4" s="7">
+        <v>400</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="D5" s="7">
+        <v>32</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="H5" s="7">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="D6" s="7">
+        <v>32</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="H6" s="7">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A7" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="D7" s="7">
+        <v>32</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="H7" s="7">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A8" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="D8" s="7">
+        <v>32</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="H8" s="7">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A9" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="D9" s="7">
+        <v>32</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="H9" s="7">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A10" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="D10" s="7">
+        <v>100</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="H10" s="7">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A11" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="D11" s="7">
+        <v>23</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="F11" s="7">
+        <v>318500</v>
+      </c>
+      <c r="H11" s="7">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A12" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="D12" s="7">
+        <v>23</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="G12" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="H12" s="7">
+        <v>400</v>
+      </c>
+      <c r="I12" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A13" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>150</v>
+      </c>
+      <c r="D13" s="7">
+        <v>23</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="G13" s="7">
+        <v>1234556</v>
+      </c>
+      <c r="H13" s="7">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A14" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="D14" s="7">
+        <v>23</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="G14" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="H14" s="7">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A15" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="D15" s="7">
+        <v>23</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="F15" s="7">
+        <v>3155</v>
+      </c>
+      <c r="H15" s="7">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A16" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="D16" s="7">
+        <v>23</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="H16" s="7">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A17" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="D17" s="7">
+        <v>23</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="H17" s="7">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A18" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="D18" s="7">
+        <v>23</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="H18" s="7">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A19" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="D19" s="7">
+        <v>61</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="H19" s="7">
+        <v>200</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B8" r:id="rId1" xr:uid="{DC99BC7A-64BD-4ED5-9C5D-734887CE02DD}"/>
+    <hyperlink ref="G12" r:id="rId2" xr:uid="{66B6DC06-85C3-48BE-840E-39D652EEFB25}"/>
+    <hyperlink ref="G13" r:id="rId3" display="special#@$" xr:uid="{0A382287-762C-4B07-A1D0-8EA6391421EB}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId4"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22757D4C-F080-489E-A73F-2A896567495D}">
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="76.36328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.6328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.6328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.81640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.1796875" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="8.90625" style="1"/>
+    <col min="1" max="1" width="76.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1530,7 +2246,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>29</v>
       </c>
@@ -1547,7 +2263,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>30</v>
       </c>
@@ -1561,7 +2277,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>36</v>
       </c>
@@ -1569,7 +2285,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>31</v>
       </c>
@@ -1586,7 +2302,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>26</v>
       </c>
@@ -1603,7 +2319,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>25</v>
       </c>
@@ -1620,7 +2336,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>27</v>
       </c>
@@ -1637,15 +2353,15 @@
         <v>401</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>28</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>56</v>
+        <v>168</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>57</v>
+        <v>169</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>6</v>
@@ -1663,16 +2379,16 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{458CF4CC-71E0-4C0E-BD04-A3D022DB64FD}">
   <dimension ref="A1:E8"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="67.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.90625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.90625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="67.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.88671875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1689,7 +2405,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>37</v>
       </c>
@@ -1706,7 +2422,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>42</v>
       </c>
@@ -1720,7 +2436,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>43</v>
       </c>
@@ -1737,7 +2453,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>38</v>
       </c>
@@ -1754,12 +2470,12 @@
         <v>400</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>39</v>
       </c>
       <c r="C6" t="s">
-        <v>60</v>
+        <v>170</v>
       </c>
       <c r="D6" t="s">
         <v>6</v>
@@ -1768,7 +2484,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>32</v>
       </c>
@@ -1785,15 +2501,15 @@
         <v>401</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>40</v>
       </c>
       <c r="B8" t="s">
-        <v>58</v>
+        <v>171</v>
       </c>
       <c r="C8" t="s">
-        <v>59</v>
+        <v>172</v>
       </c>
       <c r="D8" t="s">
         <v>6</v>
@@ -1805,4 +2521,522 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E0C88B7-415D-4393-A5FF-4B4B6EE343B5}">
+  <dimension ref="A1:I25"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="80.109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.33203125" style="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.5546875" style="6" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.5546875" style="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.88671875" style="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.33203125" style="6" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.44140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="8.88671875" style="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A2" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="D2" s="6">
+        <v>10</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="H2" s="6">
+        <v>201</v>
+      </c>
+      <c r="I2" s="9">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A3" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="H3" s="6">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="D4" s="6">
+        <v>10</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F4" s="6">
+        <v>3310</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="H4" s="6">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="D5" s="6">
+        <v>10</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F5" s="6">
+        <v>3310</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="H5" s="6">
+        <v>400</v>
+      </c>
+      <c r="I5" s="9">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="D6" s="6">
+        <v>10</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="H6" s="6">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A7" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D7" s="6">
+        <v>10</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="H7" s="6">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A8" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="D8" s="6">
+        <v>10</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="H8" s="6">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A9" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="D9" s="6">
+        <v>10</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="H9" s="6">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" s="10" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="D10" s="10">
+        <v>10</v>
+      </c>
+      <c r="E10" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="H10" s="10">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A11" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="D11" s="6">
+        <v>10</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="H11" s="6">
+        <v>400</v>
+      </c>
+      <c r="I11" s="9">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A12" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="D12" s="6">
+        <v>10</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="H12" s="6">
+        <v>400</v>
+      </c>
+      <c r="I12" s="9">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A13" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="D13" s="6">
+        <v>10</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="H13" s="6">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A14" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="D14" s="6">
+        <v>10</v>
+      </c>
+      <c r="E14" s="6">
+        <v>12367</v>
+      </c>
+      <c r="H14" s="6">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A15" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="D15" s="6">
+        <v>10</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="H15" s="6">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A16" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="H16" s="6">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A17" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="D17" s="6">
+        <v>0.5</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="H17" s="6">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A18" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="D18" s="6">
+        <v>100</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="H18" s="6">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A19" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="D19" s="6">
+        <v>10</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F19" s="6">
+        <v>3155</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="H19" s="6">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A20" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="D20" s="6">
+        <v>10</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F20" s="6">
+        <v>318500</v>
+      </c>
+      <c r="G20" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="H20" s="6">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A21" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="D21" s="6">
+        <v>10</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="H21" s="6">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A22" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="D22" s="6">
+        <v>10</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="H22" s="6">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A23" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="D23" s="6">
+        <v>10</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="H23" s="6">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A24" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="D24" s="6">
+        <v>50</v>
+      </c>
+      <c r="E24" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="H24" s="6">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A25" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="D25" s="6">
+        <v>20</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="H25" s="6">
+        <v>201</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E15" r:id="rId1" display="$#@" xr:uid="{FD56A151-1378-44EB-AF34-1C9460C6010D}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Updated logger messages for logs and new test data file
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/Team5Data.xlsx
+++ b/src/test/resources/testData/Team5Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sudhi\IdeaProjects\APITesters_Team05\src\test\resources\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17D83EB8-95B5-4D45-8EEF-24BFF3D3E1D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42A4B9D6-37DB-47E1-BA7E-712A19A09224}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="5" activeTab="8" xr2:uid="{E075535D-C164-41C6-889D-32DAEADAA696}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E075535D-C164-41C6-889D-32DAEADAA696}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="8" r:id="rId1"/>
@@ -18,9 +18,9 @@
     <sheet name="ForgotPassword" sheetId="9" r:id="rId3"/>
     <sheet name="CreateProgram" sheetId="2" r:id="rId4"/>
     <sheet name="ProgramSetupsheetname" sheetId="7" r:id="rId5"/>
-    <sheet name="UpdateBatchbyBatchId" sheetId="11" r:id="rId6"/>
-    <sheet name="UpdateProgramById" sheetId="3" r:id="rId7"/>
-    <sheet name="UpdateProgramByName" sheetId="6" r:id="rId8"/>
+    <sheet name="UpdateProgramById" sheetId="3" r:id="rId6"/>
+    <sheet name="UpdateProgramByName" sheetId="6" r:id="rId7"/>
+    <sheet name="UpdateBatchbyBatchId" sheetId="11" r:id="rId8"/>
     <sheet name="CreateBatch" sheetId="14" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -506,68 +506,68 @@
     <t>speci&amp;l#@$</t>
   </si>
   <si>
-    <t>bug</t>
-  </si>
-  <si>
     <t>200 ok bug update with associate pgm name of pgm id</t>
   </si>
   <si>
-    <t>TeamFive@123</t>
+    <t>bug 404</t>
+  </si>
+  <si>
+    <t>Valid Email</t>
   </si>
   <si>
     <t>TeamFive@125</t>
   </si>
   <si>
-    <t>Valid Email</t>
-  </si>
-  <si>
-    <t>Live on Mars safelyop</t>
-  </si>
-  <si>
-    <t>MarsLifePrepop</t>
-  </si>
-  <si>
-    <t>StarVoyagersop</t>
-  </si>
-  <si>
-    <t>BattleArenaop</t>
-  </si>
-  <si>
-    <t>Fight to surviveop</t>
-  </si>
-  <si>
-    <t>Amindb Testsop</t>
-  </si>
-  <si>
-    <t>Care for unicornop</t>
-  </si>
-  <si>
-    <t>UnicornCareop</t>
-  </si>
-  <si>
-    <t>DeleteNamePhoenixop</t>
-  </si>
-  <si>
-    <t>Delete test id caseop</t>
-  </si>
-  <si>
-    <t>DeleteByIdDragonop</t>
-  </si>
-  <si>
-    <t>test-abc_18</t>
-  </si>
-  <si>
-    <t>test-ab78</t>
-  </si>
-  <si>
-    <t>test-ab_38</t>
+    <t>TeamFive@124</t>
+  </si>
+  <si>
+    <t>Live on Mars safely</t>
+  </si>
+  <si>
+    <t>MarsLifePrep</t>
+  </si>
+  <si>
+    <t>StarVoyagers</t>
+  </si>
+  <si>
+    <t>BattleArena</t>
+  </si>
+  <si>
+    <t>Fight to survive</t>
+  </si>
+  <si>
+    <t>UnicornCare</t>
+  </si>
+  <si>
+    <t>Care for unicorn</t>
+  </si>
+  <si>
+    <t>DeleteByIdDragon</t>
+  </si>
+  <si>
+    <t>Delete test id case</t>
+  </si>
+  <si>
+    <t>DeleteNamePhoenix</t>
+  </si>
+  <si>
+    <t>Amindb Testa</t>
+  </si>
+  <si>
+    <t>test-abc_85</t>
+  </si>
+  <si>
+    <t>test-ab65</t>
+  </si>
+  <si>
+    <t>test-ab_70</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -610,10 +610,17 @@
       <family val="1"/>
     </font>
     <font>
-      <sz val="7"/>
-      <color rgb="FF0451A5"/>
-      <name val="Courier New"/>
-      <family val="3"/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -690,7 +697,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -714,14 +721,11 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1060,7 +1064,7 @@
         <v>55</v>
       </c>
       <c r="B2" s="3"/>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="4" t="s">
         <v>160</v>
       </c>
       <c r="D2" s="3">
@@ -1074,7 +1078,7 @@
       <c r="B3" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="C3" s="12" t="s">
+      <c r="C3" s="4" t="s">
         <v>160</v>
       </c>
       <c r="D3" s="3">
@@ -1088,7 +1092,7 @@
       <c r="B4" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="C4" s="4" t="s">
         <v>160</v>
       </c>
       <c r="D4" s="3">
@@ -1102,7 +1106,7 @@
       <c r="B5" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="C5" s="12" t="s">
+      <c r="C5" s="4" t="s">
         <v>160</v>
       </c>
       <c r="D5" s="3">
@@ -1116,7 +1120,7 @@
       <c r="B6" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="C6" s="12" t="s">
+      <c r="C6" s="4" t="s">
         <v>160</v>
       </c>
       <c r="D6" s="3">
@@ -1148,8 +1152,8 @@
       <c r="D8" s="3">
         <v>401</v>
       </c>
-      <c r="E8" s="11" t="s">
-        <v>157</v>
+      <c r="E8" s="12" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
@@ -1187,7 +1191,7 @@
       <c r="B11" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="C11" s="12" t="s">
+      <c r="C11" s="4" t="s">
         <v>160</v>
       </c>
       <c r="D11" s="3">
@@ -1201,7 +1205,7 @@
       <c r="B12" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="C12" s="12" t="s">
+      <c r="C12" s="4" t="s">
         <v>160</v>
       </c>
       <c r="D12" s="3">
@@ -1215,7 +1219,7 @@
       <c r="B13" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="C13" s="12" t="s">
+      <c r="C13" s="4" t="s">
         <v>160</v>
       </c>
       <c r="D13" s="3">
@@ -1232,14 +1236,14 @@
     <hyperlink ref="B10" r:id="rId6" xr:uid="{D6942936-5D52-4C4A-8ECA-9DE8722DC4E7}"/>
     <hyperlink ref="B12" r:id="rId7" xr:uid="{3C895F9A-5852-422F-BA70-9072953C0F79}"/>
     <hyperlink ref="B13" r:id="rId8" xr:uid="{76EFE8C1-C1B1-43B2-BA64-14F7AC4BAF9C}"/>
-    <hyperlink ref="C2" r:id="rId9" xr:uid="{127FD2B5-78BB-464B-A9CD-CD008DC6CD93}"/>
-    <hyperlink ref="C3" r:id="rId10" xr:uid="{8DF09848-83DE-4BBF-B1A2-1AEEA19B4346}"/>
-    <hyperlink ref="C4" r:id="rId11" xr:uid="{19881271-15CD-4524-88E0-7E1A48BEE6D7}"/>
-    <hyperlink ref="C5" r:id="rId12" xr:uid="{31DDF559-C92D-4E93-A112-5CF6787C9F78}"/>
-    <hyperlink ref="C6" r:id="rId13" xr:uid="{485AF9D4-F737-467E-9B83-4DE2D7921067}"/>
-    <hyperlink ref="C11" r:id="rId14" xr:uid="{E9BE5A0B-436B-4C8D-A311-75820BD6C958}"/>
-    <hyperlink ref="C12" r:id="rId15" xr:uid="{6642A2F1-B387-4F6D-8494-366A09C46D80}"/>
-    <hyperlink ref="C13" r:id="rId16" xr:uid="{1156645C-D24C-4677-A8E8-4489D07A92B0}"/>
+    <hyperlink ref="C2" r:id="rId9" xr:uid="{45139CDB-7F83-47D6-A63C-DDE4BE6B20C5}"/>
+    <hyperlink ref="C3" r:id="rId10" xr:uid="{F2879478-943A-4900-AA4D-6A0F629BD782}"/>
+    <hyperlink ref="C4" r:id="rId11" xr:uid="{CCF02A3F-5360-4087-813C-AD6B8EE3B51F}"/>
+    <hyperlink ref="C5" r:id="rId12" xr:uid="{EC6E90FA-7C60-4DE2-BD18-39348E83071C}"/>
+    <hyperlink ref="C6" r:id="rId13" xr:uid="{3FFC32D8-62F5-4249-92D9-65E05D257513}"/>
+    <hyperlink ref="C11" r:id="rId14" xr:uid="{47B28374-8037-45C3-BE27-6B2CBB57AA5E}"/>
+    <hyperlink ref="C12" r:id="rId15" xr:uid="{F1A96C9A-DAF6-48AB-8349-7FBF0C5754BD}"/>
+    <hyperlink ref="C13" r:id="rId16" xr:uid="{41029459-D036-48A2-BDE2-BB4074D70C0B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1272,7 +1276,7 @@
         <v>73</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="D2" s="3">
         <v>200</v>
@@ -1286,7 +1290,7 @@
         <v>76</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="D3" s="3">
         <v>400</v>
@@ -1314,7 +1318,7 @@
         <v>73</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="D5" s="3">
         <v>404</v>
@@ -1328,7 +1332,7 @@
         <v>73</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="D6" s="3">
         <v>405</v>
@@ -1342,7 +1346,7 @@
         <v>73</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="D7" s="3">
         <v>401</v>
@@ -1362,18 +1366,18 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C4" r:id="rId1" display="TeamFive@123" xr:uid="{AEDF5809-446B-449F-BA4B-A222C3D449A1}"/>
-    <hyperlink ref="B2" r:id="rId2" xr:uid="{EB1FE2E9-B2D8-4457-9393-B039145DF400}"/>
-    <hyperlink ref="B3" r:id="rId3" xr:uid="{C9CE5294-9DE5-4433-8E4C-2466145586EF}"/>
-    <hyperlink ref="B4" r:id="rId4" xr:uid="{052FE08C-B5BB-4AEC-B1E4-D5E5C39AE2DF}"/>
-    <hyperlink ref="B5" r:id="rId5" xr:uid="{146FF6F4-CFA0-4965-BB12-16ED707B7AFF}"/>
-    <hyperlink ref="B6" r:id="rId6" xr:uid="{C10FE077-11C5-4888-85F2-476E58BD487E}"/>
-    <hyperlink ref="B7" r:id="rId7" xr:uid="{34847948-15D7-4525-A5B9-0610F9EDA075}"/>
-    <hyperlink ref="C2" r:id="rId8" xr:uid="{D5776F13-F123-4867-B73F-0FD7E5F4C73B}"/>
-    <hyperlink ref="C3" r:id="rId9" xr:uid="{D352CC11-255C-46C6-982D-C549B1581CEF}"/>
-    <hyperlink ref="C5" r:id="rId10" xr:uid="{9CA76A89-3119-49B8-BB35-B0EF3178D561}"/>
-    <hyperlink ref="C6" r:id="rId11" xr:uid="{06BEA948-B30F-4124-AEC4-D20FF720AF46}"/>
-    <hyperlink ref="C7" r:id="rId12" xr:uid="{AE33B4A3-38EB-4675-B6BD-F9375CD09E48}"/>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{EB1FE2E9-B2D8-4457-9393-B039145DF400}"/>
+    <hyperlink ref="B3" r:id="rId2" xr:uid="{C9CE5294-9DE5-4433-8E4C-2466145586EF}"/>
+    <hyperlink ref="B4" r:id="rId3" xr:uid="{052FE08C-B5BB-4AEC-B1E4-D5E5C39AE2DF}"/>
+    <hyperlink ref="B5" r:id="rId4" xr:uid="{146FF6F4-CFA0-4965-BB12-16ED707B7AFF}"/>
+    <hyperlink ref="B6" r:id="rId5" xr:uid="{C10FE077-11C5-4888-85F2-476E58BD487E}"/>
+    <hyperlink ref="B7" r:id="rId6" xr:uid="{34847948-15D7-4525-A5B9-0610F9EDA075}"/>
+    <hyperlink ref="C4" r:id="rId7" display="TeamFive@123" xr:uid="{AEDF5809-446B-449F-BA4B-A222C3D449A1}"/>
+    <hyperlink ref="C7" r:id="rId8" xr:uid="{C62C0FC6-1D60-4EFE-9F06-C223C393FD29}"/>
+    <hyperlink ref="C6" r:id="rId9" xr:uid="{CE3A4846-EE1A-49C1-9620-F28CEEE270FC}"/>
+    <hyperlink ref="C5" r:id="rId10" xr:uid="{DF1F7E3C-05D9-4471-A6E2-C9B25D62082F}"/>
+    <hyperlink ref="C3" r:id="rId11" xr:uid="{AFAF4C99-8411-4274-8FB0-46A04E3400A8}"/>
+    <hyperlink ref="C2" r:id="rId12" xr:uid="{7BC4345E-DECE-45FA-A399-7A485906A19D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1463,10 +1467,10 @@
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="3" t="s">
-        <v>161</v>
-      </c>
-      <c r="B8" s="13" t="s">
+      <c r="A8" t="s">
+        <v>159</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>73</v>
       </c>
       <c r="C8" s="3">
@@ -1497,6 +1501,7 @@
   <hyperlinks>
     <hyperlink ref="B7" r:id="rId1" display="mailto:notfound@mail.com" xr:uid="{CDB8C9B5-8B80-4157-848A-E22D2B3C197C}"/>
     <hyperlink ref="B3" r:id="rId2" xr:uid="{49CEACEE-7FC1-4CA9-AE76-D1F4F824CF67}"/>
+    <hyperlink ref="B8" r:id="rId3" xr:uid="{EE5510AE-E412-4ADD-97EA-7FCE50C7E554}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1801,6 +1806,313 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22757D4C-F080-489E-A73F-2A896567495D}">
+  <dimension ref="A1:E9"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="76.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="8.88671875" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" s="1">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E3" s="1">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E4" s="1">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E5" s="1">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E6" s="1">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E7" s="1">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E8" s="1">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E9" s="1">
+        <v>200</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{458CF4CC-71E0-4C0E-BD04-A3D022DB64FD}">
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="67.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B3" t="s">
+        <v>34</v>
+      </c>
+      <c r="D3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E3">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C4" t="s">
+        <v>35</v>
+      </c>
+      <c r="D4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>38</v>
+      </c>
+      <c r="B5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C5" t="s">
+        <v>35</v>
+      </c>
+      <c r="D5" t="s">
+        <v>6</v>
+      </c>
+      <c r="E5">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C6" t="s">
+        <v>171</v>
+      </c>
+      <c r="D6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E6">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B7" t="s">
+        <v>34</v>
+      </c>
+      <c r="C7" t="s">
+        <v>35</v>
+      </c>
+      <c r="D7" t="s">
+        <v>6</v>
+      </c>
+      <c r="E7">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B8" t="s">
+        <v>170</v>
+      </c>
+      <c r="C8" t="s">
+        <v>169</v>
+      </c>
+      <c r="D8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E8">
+        <v>200</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D8C71BF-CB4E-4334-8784-890AB6A8A9AA}">
   <dimension ref="A1:I19"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
@@ -1886,7 +2198,7 @@
       <c r="H4" s="7">
         <v>400</v>
       </c>
-      <c r="I4" s="7" t="s">
+      <c r="I4" s="11" t="s">
         <v>151</v>
       </c>
     </row>
@@ -2055,8 +2367,8 @@
       <c r="H12" s="7">
         <v>400</v>
       </c>
-      <c r="I12" s="7" t="s">
-        <v>158</v>
+      <c r="I12" s="11" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
@@ -2099,7 +2411,7 @@
         <v>6</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="H14" s="7">
         <v>200</v>
@@ -2213,313 +2525,6 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId4"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22757D4C-F080-489E-A73F-2A896567495D}">
-  <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="76.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="8.88671875" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E2" s="1">
-        <v>404</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E3" s="1">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="E4" s="1">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E5" s="1">
-        <v>404</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E6" s="1">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E7" s="1">
-        <v>404</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E8" s="1">
-        <v>401</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E9" s="1">
-        <v>200</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{458CF4CC-71E0-4C0E-BD04-A3D022DB64FD}">
-  <dimension ref="A1:E8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="67.77734375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E2">
-        <v>404</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>42</v>
-      </c>
-      <c r="B3" t="s">
-        <v>34</v>
-      </c>
-      <c r="D3" t="s">
-        <v>6</v>
-      </c>
-      <c r="E3">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>43</v>
-      </c>
-      <c r="B4" t="s">
-        <v>34</v>
-      </c>
-      <c r="C4" t="s">
-        <v>35</v>
-      </c>
-      <c r="D4" t="s">
-        <v>14</v>
-      </c>
-      <c r="E4">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>38</v>
-      </c>
-      <c r="B5" t="s">
-        <v>41</v>
-      </c>
-      <c r="C5" t="s">
-        <v>35</v>
-      </c>
-      <c r="D5" t="s">
-        <v>6</v>
-      </c>
-      <c r="E5">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>39</v>
-      </c>
-      <c r="C6" t="s">
-        <v>170</v>
-      </c>
-      <c r="D6" t="s">
-        <v>6</v>
-      </c>
-      <c r="E6">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>32</v>
-      </c>
-      <c r="B7" t="s">
-        <v>34</v>
-      </c>
-      <c r="C7" t="s">
-        <v>35</v>
-      </c>
-      <c r="D7" t="s">
-        <v>6</v>
-      </c>
-      <c r="E7">
-        <v>401</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>40</v>
-      </c>
-      <c r="B8" t="s">
-        <v>171</v>
-      </c>
-      <c r="C8" t="s">
-        <v>172</v>
-      </c>
-      <c r="D8" t="s">
-        <v>6</v>
-      </c>
-      <c r="E8">
-        <v>200</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 

</xml_diff>